<commit_message>
Update annotations and flags in Zive data JSON files
- Changed flags from "PSEUDO_ANNOTATED" to "FULLY_ANNOTATED_PROFESSIONALLY" and added "FOR_EXTERNAL_ANNOTATING" in multiple JSON files.
- Updated comments to provide clearer descriptions in the annotation data.
- Adjusted rpeak annotation counts and values for various samples to reflect accurate annotations.
- Modified sample indices and annotation values to ensure consistency across datasets.
- Deleted outdated Excel files and added new versions to maintain up-to-date records.
- Updated the shell script to streamline the process of adding ML noises and annotations.
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/08_Anotacijos_logai/08_Anotavimo_logas.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/08_Anotacijos_logai/08_Anotavimo_logas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\AnotacijosLogai\08_Anotacijos_logai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6134C10E-E57A-46A3-BB70-69750A87E702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75B8887-C723-44A5-AA25-83F782E85AD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-260" yWindow="960" windowWidth="18600" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="18600" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="logas" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="47">
   <si>
     <t>basename</t>
   </si>
@@ -171,6 +171,12 @@
   </si>
   <si>
     <t>1025_2</t>
+  </si>
+  <si>
+    <t>Ž:  Kelis kartus po skilvelinės ekstrasistolės šiame įraše stebime vadinamus "fusion beat" (susiliejęs kompleksas). Jį lemia tai, jog skilvelių depoliarizaciją lemia tiek neseniai buvusi skilvelinė ekstrasistolė, tiek iš sinusinio mazgo atėjęs impulsas ir šios dvi skilvelio aktyvacijos susilieja, todėl keičia morfologiją, palyginus su įprastu sinusiniu kompleksu, tačiau nėra platus kaip skilvelinė ekstrasistolė. Šiuo atveju tai nėra nei skilvelinė, nei prieširdinė ekstrasistolės, nei normalus QRS kompleksas. Tam, kad neklaidinti algoritmo pažymėjau juos U raide.</t>
+  </si>
+  <si>
+    <t>1643055.090</t>
   </si>
 </sst>
 </file>
@@ -224,7 +230,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -262,11 +268,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -291,6 +308,13 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -572,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.81640625" bestFit="1" customWidth="1"/>
@@ -655,14 +679,16 @@
       <c r="D2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" s="4"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="G2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="4"/>
+      <c r="H2" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="6" t="s">
@@ -677,6 +703,9 @@
       <c r="N2" t="s">
         <v>28</v>
       </c>
+      <c r="O2" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3">
@@ -691,14 +720,16 @@
       <c r="D3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" s="4"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="G3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="4"/>
+      <c r="H3" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="6" t="s">
@@ -728,14 +759,16 @@
       <c r="D4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4" s="4"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="G4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="4"/>
+      <c r="H4" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="6"/>
@@ -763,14 +796,16 @@
       <c r="D5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F5" s="4"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="G5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H5" s="4"/>
+      <c r="H5" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="6" t="s">
@@ -800,14 +835,16 @@
       <c r="D6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" s="4"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="G6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H6" s="4"/>
+      <c r="H6" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="6" t="s">
@@ -837,14 +874,16 @@
       <c r="D7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F7" s="4"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="G7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="4"/>
+      <c r="H7" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="6" t="s">
@@ -874,14 +913,16 @@
       <c r="D8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F8" s="4"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="G8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="4"/>
+      <c r="H8" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="6" t="s">
@@ -896,6 +937,26 @@
       <c r="N8" t="str">
         <f>""</f>
         <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A9" s="11">
+        <v>8</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>